<commit_message>
Refine checkout task language and business answers
</commit_message>
<xml_diff>
--- a/artifacts/任务规格转化.xlsx
+++ b/artifacts/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R542f27276c1948cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R731fa76fee1f445c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -471,34 +471,26 @@
     </x:row>
     <x:row r="15" ht="54" customHeight="1">
       <x:c r="A15" s="14" t="str">
-        <x:v>失败收口</x:v>
+        <x:v>完成条件</x:v>
       </x:c>
       <x:c r="B15" s="21" t="str">
-        <x:v>tools/run-task.mjs调用Playwright；任一测试失败时清理本轮reports、evidence、test-results和临时运行目录，避免旧结果被误用</x:v>
+        <x:v>npm run test:e2e使用锁定版本的Playwright与Chromium完成所有场景，四份报表与逐场景证据相互对应</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="52" customHeight="1">
       <x:c r="A16" s="14" t="str">
-        <x:v>完成条件</x:v>
+        <x:v>工作要点</x:v>
       </x:c>
       <x:c r="B16" s="21" t="str">
-        <x:v>npm run test:e2e可以在Windows11原生环境中使用锁定版本的Playwright与Chromium完成回归，四份报表与十二份证据相互对应，同一输入重复运行的结构化语义一致</x:v>
+        <x:v>读取三类业务输入；稳定定位；route响应序列；支付方式交互；最终请求参数；浏览器时间；焦点断言；trace与截图可用性</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="52" customHeight="1">
       <x:c r="A17" s="14" t="str">
-        <x:v>可验证点</x:v>
+        <x:v>评分边界</x:v>
       </x:c>
       <x:c r="B17" s="21" t="str">
-        <x:v>真实Chromium进程；三类输入读取；稳定定位；route响应序列；支付方式交互；最终请求参数；浏览器时间；焦点断言；trace与截图可用性；失败清理</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="52" customHeight="1">
-      <x:c r="A18" s="14" t="str">
-        <x:v>不适合作为评分点的内容</x:v>
-      </x:c>
-      <x:c r="B18" s="21" t="str">
-        <x:v>代码缩进、注释数量、内部函数名、测试标题措辞、CSV行顺序、JSON键顺序、trace与截图字节哈希及不改变业务结果的附加说明文件</x:v>
+        <x:v>代码缩进、注释数量、内部函数名、测试标题措辞、CSV行顺序、JSON键顺序及不改变业务结果的附加说明文件不计分</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>